<commit_message>
Add South Korea to oil price CPI/PPI impact analysis
South Korea results (per 10% oil price increase):
- CPI: +0.18pp (Direct: 0.12pp / 67%, Indirect: 0.06pp / 33%)
- PPI: +0.50pp (Direct: 0.35pp / 70%, Indirect: 0.15pp / 30%)

Key Korea-specific factors:
- Highest oil intensity in OECD (5.63 bbl per $10K GDP)
- Renewable energy only 9% (vs OECD avg 33%)
- 70%+ oil imports through Strait of Hormuz
- CPI petroleum weight ~5.2% (2022 rebase by Statistics Korea)
- Manufacturing-heavy economy amplifies PPI sensitivity

Sources: KDI (2024), Hyundai Research Institute (2024),
J. Asian Economics Vol.96 (2025), Statistics Korea (2023),
Citibank (2026)

Co-authored-by: Zzxmh <Zzxmh@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/oil_price_impact_analysis.xlsx
+++ b/output/oil_price_impact_analysis.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -727,6 +727,72 @@
       </c>
       <c r="I9" t="n">
         <v>30.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CPI</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>35</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H10" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I10" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PPI</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>13</v>
+      </c>
+      <c r="D11" t="n">
+        <v>50</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H11" t="n">
+        <v>70</v>
+      </c>
+      <c r="I11" t="n">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -740,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1131,7 +1197,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1140,39 +1206,39 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3.5</v>
+        <v>5.2</v>
       </c>
       <c r="D10" t="n">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E10" t="n">
-        <v>0.36</v>
+        <v>0.12</v>
       </c>
       <c r="F10" t="n">
-        <v>0.09</v>
+        <v>0.06</v>
       </c>
       <c r="G10" t="n">
-        <v>0.45</v>
+        <v>0.18</v>
       </c>
       <c r="H10" t="n">
-        <v>80</v>
+        <v>66.7</v>
       </c>
       <c r="I10" t="n">
-        <v>20</v>
+        <v>33.3</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Moderate (+30%)</t>
+          <t>Mild (+10%)</t>
         </is>
       </c>
       <c r="K10" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1181,39 +1247,39 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D11" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="E11" t="n">
-        <v>0.75</v>
+        <v>0.35</v>
       </c>
       <c r="F11" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="G11" t="n">
-        <v>1.05</v>
+        <v>0.5</v>
       </c>
       <c r="H11" t="n">
-        <v>71.40000000000001</v>
+        <v>70</v>
       </c>
       <c r="I11" t="n">
-        <v>28.6</v>
+        <v>30</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Moderate (+30%)</t>
+          <t>Mild (+10%)</t>
         </is>
       </c>
       <c r="K11" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>China</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1222,25 +1288,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6.5</v>
+        <v>3.5</v>
       </c>
       <c r="D12" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E12" t="n">
-        <v>0.3</v>
+        <v>0.36</v>
       </c>
       <c r="F12" t="n">
-        <v>0.15</v>
+        <v>0.09</v>
       </c>
       <c r="G12" t="n">
         <v>0.45</v>
       </c>
       <c r="H12" t="n">
-        <v>66.7</v>
+        <v>80</v>
       </c>
       <c r="I12" t="n">
-        <v>33.3</v>
+        <v>20</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1254,7 +1320,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>China</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1263,25 +1329,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10.5</v>
+        <v>12</v>
       </c>
       <c r="D13" t="n">
-        <v>55.00000000000001</v>
+        <v>25</v>
       </c>
       <c r="E13" t="n">
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
       <c r="F13" t="n">
         <v>0.3</v>
       </c>
       <c r="G13" t="n">
-        <v>1.2</v>
+        <v>1.05</v>
       </c>
       <c r="H13" t="n">
-        <v>75</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>25</v>
+        <v>28.6</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1295,7 +1361,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1304,25 +1370,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="D14" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="E14" t="n">
-        <v>0.18</v>
+        <v>0.3</v>
       </c>
       <c r="F14" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3</v>
+        <v>0.45</v>
       </c>
       <c r="H14" t="n">
-        <v>60</v>
+        <v>66.7</v>
       </c>
       <c r="I14" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1336,7 +1402,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1345,25 +1411,25 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14</v>
+        <v>10.5</v>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="E15" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G15" t="n">
         <v>1.2</v>
       </c>
-      <c r="F15" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="G15" t="n">
-        <v>1.65</v>
-      </c>
       <c r="H15" t="n">
-        <v>72.7</v>
+        <v>75</v>
       </c>
       <c r="I15" t="n">
-        <v>27.3</v>
+        <v>25</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1377,7 +1443,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1386,19 +1452,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9.67</v>
+        <v>7</v>
       </c>
       <c r="D16" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E16" t="n">
-        <v>0.36</v>
+        <v>0.18</v>
       </c>
       <c r="F16" t="n">
-        <v>0.24</v>
+        <v>0.12</v>
       </c>
       <c r="G16" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="H16" t="n">
         <v>60</v>
@@ -1418,7 +1484,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1427,25 +1493,25 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>15.5</v>
+        <v>14</v>
       </c>
       <c r="D17" t="n">
-        <v>55.00000000000001</v>
+        <v>50</v>
       </c>
       <c r="E17" t="n">
-        <v>1.35</v>
+        <v>1.2</v>
       </c>
       <c r="F17" t="n">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="G17" t="n">
-        <v>1.95</v>
+        <v>1.65</v>
       </c>
       <c r="H17" t="n">
-        <v>69.2</v>
+        <v>72.7</v>
       </c>
       <c r="I17" t="n">
-        <v>30.8</v>
+        <v>27.3</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1459,7 +1525,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1468,39 +1534,39 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3.5</v>
+        <v>9.67</v>
       </c>
       <c r="D18" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E18" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G18" t="n">
         <v>0.6</v>
       </c>
-      <c r="F18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0.75</v>
-      </c>
       <c r="H18" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="I18" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Severe (+50%)</t>
+          <t>Moderate (+30%)</t>
         </is>
       </c>
       <c r="K18" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1509,39 +1575,39 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>12</v>
+        <v>15.5</v>
       </c>
       <c r="D19" t="n">
-        <v>25</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="E19" t="n">
-        <v>1.25</v>
+        <v>1.35</v>
       </c>
       <c r="F19" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="G19" t="n">
-        <v>1.75</v>
+        <v>1.95</v>
       </c>
       <c r="H19" t="n">
-        <v>71.40000000000001</v>
+        <v>69.2</v>
       </c>
       <c r="I19" t="n">
-        <v>28.6</v>
+        <v>30.8</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Severe (+50%)</t>
+          <t>Moderate (+30%)</t>
         </is>
       </c>
       <c r="K19" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1550,19 +1616,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>6.5</v>
+        <v>5.2</v>
       </c>
       <c r="D20" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="E20" t="n">
-        <v>0.5</v>
+        <v>0.36</v>
       </c>
       <c r="F20" t="n">
-        <v>0.25</v>
+        <v>0.18</v>
       </c>
       <c r="G20" t="n">
-        <v>0.75</v>
+        <v>0.54</v>
       </c>
       <c r="H20" t="n">
         <v>66.7</v>
@@ -1572,17 +1638,17 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Severe (+50%)</t>
+          <t>Moderate (+30%)</t>
         </is>
       </c>
       <c r="K20" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1591,39 +1657,39 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>10.5</v>
+        <v>13</v>
       </c>
       <c r="D21" t="n">
-        <v>55.00000000000001</v>
+        <v>50</v>
       </c>
       <c r="E21" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G21" t="n">
         <v>1.5</v>
       </c>
-      <c r="F21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G21" t="n">
-        <v>2</v>
-      </c>
       <c r="H21" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="I21" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Severe (+50%)</t>
+          <t>Moderate (+30%)</t>
         </is>
       </c>
       <c r="K21" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1632,25 +1698,25 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>7</v>
+        <v>3.5</v>
       </c>
       <c r="D22" t="n">
+        <v>43</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H22" t="n">
+        <v>80</v>
+      </c>
+      <c r="I22" t="n">
         <v>20</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H22" t="n">
-        <v>60</v>
-      </c>
-      <c r="I22" t="n">
-        <v>40</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1664,7 +1730,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1673,25 +1739,25 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D23" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>1.25</v>
       </c>
       <c r="F23" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="G23" t="n">
-        <v>2.75</v>
+        <v>1.75</v>
       </c>
       <c r="H23" t="n">
-        <v>72.7</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="I23" t="n">
-        <v>27.3</v>
+        <v>28.6</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1705,7 +1771,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1714,25 +1780,25 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>9.67</v>
+        <v>6.5</v>
       </c>
       <c r="D24" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="F24" t="n">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="G24" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="H24" t="n">
-        <v>60</v>
+        <v>66.7</v>
       </c>
       <c r="I24" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1746,7 +1812,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1755,25 +1821,25 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>15.5</v>
+        <v>10.5</v>
       </c>
       <c r="D25" t="n">
         <v>55.00000000000001</v>
       </c>
       <c r="E25" t="n">
-        <v>2.25</v>
+        <v>1.5</v>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G25" t="n">
-        <v>3.25</v>
+        <v>2</v>
       </c>
       <c r="H25" t="n">
-        <v>69.2</v>
+        <v>75</v>
       </c>
       <c r="I25" t="n">
-        <v>30.8</v>
+        <v>25</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -1787,7 +1853,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1796,39 +1862,39 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3.5</v>
+        <v>7</v>
       </c>
       <c r="D26" t="n">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="E26" t="n">
-        <v>1.2</v>
+        <v>0.3</v>
       </c>
       <c r="F26" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="G26" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="H26" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="I26" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Extreme (+100%)</t>
+          <t>Severe (+50%)</t>
         </is>
       </c>
       <c r="K26" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1837,39 +1903,39 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D27" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="E27" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="G27" t="n">
-        <v>3.5</v>
+        <v>2.75</v>
       </c>
       <c r="H27" t="n">
-        <v>71.40000000000001</v>
+        <v>72.7</v>
       </c>
       <c r="I27" t="n">
-        <v>28.6</v>
+        <v>27.3</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Extreme (+100%)</t>
+          <t>Severe (+50%)</t>
         </is>
       </c>
       <c r="K27" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1878,39 +1944,39 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>6.5</v>
+        <v>9.67</v>
       </c>
       <c r="D28" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E28" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G28" t="n">
         <v>1</v>
       </c>
-      <c r="F28" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G28" t="n">
-        <v>1.5</v>
-      </c>
       <c r="H28" t="n">
-        <v>66.7</v>
+        <v>60</v>
       </c>
       <c r="I28" t="n">
-        <v>33.3</v>
+        <v>40</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Extreme (+100%)</t>
+          <t>Severe (+50%)</t>
         </is>
       </c>
       <c r="K28" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1919,39 +1985,39 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>10.5</v>
+        <v>15.5</v>
       </c>
       <c r="D29" t="n">
         <v>55.00000000000001</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>2.25</v>
       </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>4</v>
+        <v>3.25</v>
       </c>
       <c r="H29" t="n">
-        <v>75</v>
+        <v>69.2</v>
       </c>
       <c r="I29" t="n">
-        <v>25</v>
+        <v>30.8</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Extreme (+100%)</t>
+          <t>Severe (+50%)</t>
         </is>
       </c>
       <c r="K29" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1960,39 +2026,39 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7</v>
+        <v>5.2</v>
       </c>
       <c r="D30" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="E30" t="n">
         <v>0.6</v>
       </c>
       <c r="F30" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G30" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="H30" t="n">
-        <v>60</v>
+        <v>66.7</v>
       </c>
       <c r="I30" t="n">
-        <v>40</v>
+        <v>33.3</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Extreme (+100%)</t>
+          <t>Severe (+50%)</t>
         </is>
       </c>
       <c r="K30" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2001,39 +2067,39 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D31" t="n">
         <v>50</v>
       </c>
       <c r="E31" t="n">
-        <v>4</v>
+        <v>1.75</v>
       </c>
       <c r="F31" t="n">
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="G31" t="n">
-        <v>5.5</v>
+        <v>2.5</v>
       </c>
       <c r="H31" t="n">
-        <v>72.7</v>
+        <v>70</v>
       </c>
       <c r="I31" t="n">
-        <v>27.3</v>
+        <v>30</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Extreme (+100%)</t>
+          <t>Severe (+50%)</t>
         </is>
       </c>
       <c r="K31" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2042,25 +2108,25 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>9.67</v>
+        <v>3.5</v>
       </c>
       <c r="D32" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E32" t="n">
         <v>1.2</v>
       </c>
       <c r="F32" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="G32" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="H32" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="I32" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -2074,41 +2140,369 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>PPI</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>12</v>
+      </c>
+      <c r="D33" t="n">
+        <v>25</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H33" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I33" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Extreme (+100%)</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>CPI</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D34" t="n">
+        <v>45</v>
+      </c>
+      <c r="E34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H34" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I34" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Extreme (+100%)</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PPI</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="D35" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="E35" t="n">
+        <v>3</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>4</v>
+      </c>
+      <c r="H35" t="n">
+        <v>75</v>
+      </c>
+      <c r="I35" t="n">
+        <v>25</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Extreme (+100%)</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>CPI</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>7</v>
+      </c>
+      <c r="D36" t="n">
+        <v>20</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G36" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" t="n">
+        <v>60</v>
+      </c>
+      <c r="I36" t="n">
+        <v>40</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Extreme (+100%)</t>
+        </is>
+      </c>
+      <c r="K36" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>PPI</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>14</v>
+      </c>
+      <c r="D37" t="n">
+        <v>50</v>
+      </c>
+      <c r="E37" t="n">
+        <v>4</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G37" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H37" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="I37" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Extreme (+100%)</t>
+        </is>
+      </c>
+      <c r="K37" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>Vietnam</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>PPI</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>CPI</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="D38" t="n">
+        <v>40</v>
+      </c>
+      <c r="E38" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H38" t="n">
+        <v>60</v>
+      </c>
+      <c r="I38" t="n">
+        <v>40</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Extreme (+100%)</t>
+        </is>
+      </c>
+      <c r="K38" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>PPI</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
         <v>15.5</v>
       </c>
-      <c r="D33" t="n">
+      <c r="D39" t="n">
         <v>55.00000000000001</v>
       </c>
-      <c r="E33" t="n">
+      <c r="E39" t="n">
         <v>4.5</v>
       </c>
-      <c r="F33" t="n">
+      <c r="F39" t="n">
         <v>2</v>
       </c>
-      <c r="G33" t="n">
+      <c r="G39" t="n">
         <v>6.5</v>
       </c>
-      <c r="H33" t="n">
+      <c r="H39" t="n">
         <v>69.2</v>
       </c>
-      <c r="I33" t="n">
+      <c r="I39" t="n">
         <v>30.8</v>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>Extreme (+100%)</t>
         </is>
       </c>
-      <c r="K33" t="n">
+      <c r="K39" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>CPI</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="D40" t="n">
+        <v>35</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H40" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="I40" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Extreme (+100%)</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>PPI</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>13</v>
+      </c>
+      <c r="D41" t="n">
+        <v>50</v>
+      </c>
+      <c r="E41" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G41" t="n">
+        <v>5</v>
+      </c>
+      <c r="H41" t="n">
+        <v>70</v>
+      </c>
+      <c r="I41" t="n">
+        <v>30</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Extreme (+100%)</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
         <v>100</v>
       </c>
     </row>
@@ -2123,7 +2517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2379,6 +2773,60 @@
         <v>0.65</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CPI</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PPI</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>13</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add detailed 100% oil price increase scenario analysis for all 5 countries
New dedicated analysis for extreme +100% oil price scenario (e.g. $70→$140/bbl):
- Non-linear amplification factor (1.15x) applied to indirect effects
- Validated against NRI Japan (+109%), Hyundai Research Korea (+114%), Fed DSGE

Results (Total with non-linear amplification):
  Country       CPI (pp)    PPI (pp)
  Vietnam       +2.120      +6.800
  South Korea   +1.890      +5.225
  USA           +1.575      +4.150
  China         +1.545      +3.650
  Japan         +1.060      +5.725

New output files:
- 100pct_effect_decomposition.png (stacked bar with uplift)
- 100pct_cpi_vs_ppi.png (horizontal comparison)
- analysis_report_100pct.txt (detailed 100% scenario report)
- Excel updated with Extreme_100pct sheet

Co-authored-by: Zzxmh <Zzxmh@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/oil_price_impact_analysis.xlsx
+++ b/output/oil_price_impact_analysis.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Baseline_10pct" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Scenario_Analysis" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Parameters" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Extreme_100pct" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Parameters" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2517,6 +2518,467 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Index</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Energy Weight (%)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Direct Effect (pp)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Indirect Linear (pp)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Indirect Amplified (pp)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Total Linear (pp)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Total Amplified (pp)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Non-linear Uplift (pp)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Direct Share (%)</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Indirect Share (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CPI</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.545</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="J2" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="K2" t="n">
+        <v>22.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PPI</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J3" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="K3" t="n">
+        <v>31.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CPI</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.575</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="J4" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>36.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PPI</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J5" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="K5" t="n">
+        <v>27.7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CPI</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>7</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="J6" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="K6" t="n">
+        <v>43.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PPI</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>14</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.725</v>
+      </c>
+      <c r="G7" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H7" t="n">
+        <v>5.725</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="J7" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="K7" t="n">
+        <v>30.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CPI</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="J8" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="K8" t="n">
+        <v>43.4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PPI</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J9" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="K9" t="n">
+        <v>33.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CPI</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="J10" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>36.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PPI</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>13</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.725</v>
+      </c>
+      <c r="G11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" t="n">
+        <v>5.225</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="J11" t="n">
+        <v>67</v>
+      </c>
+      <c r="K11" t="n">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>